<commit_message>
Add Sep 24 diagnosis, 70 new targets (50 sponsors, 20 organizers), forms and follow-up audit
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01MtBZkCZBeRKhcHJKr7GKax
</commit_message>
<xml_diff>
--- a/WAIFF_Refinement_Log.xlsx
+++ b/WAIFF_Refinement_Log.xlsx
@@ -658,7 +658,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F44"/>
+  <dimension ref="A1:F31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1422,26 +1422,230 @@
         </is>
       </c>
     </row>
-    <row r="25"/>
-    <row r="26"/>
-    <row r="27"/>
-    <row r="28"/>
-    <row r="29"/>
-    <row r="30"/>
-    <row r="31"/>
-    <row r="32"/>
-    <row r="33"/>
-    <row r="34"/>
-    <row r="35"/>
-    <row r="36"/>
-    <row r="37"/>
-    <row r="38"/>
-    <row r="39"/>
-    <row r="40"/>
-    <row r="41"/>
-    <row r="42"/>
-    <row r="43"/>
-    <row r="44"/>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>24 Sep 2026</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>Offer / product</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>Sell Cannes 2027 (6-7 Apr) + named editions to global sponsors. India edition (December) is the add-on for India-focused brands.</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>The India edition has no public date, venue or organizer, so brand teams cannot approve it. Venues replied only to sell rooms.</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>523 companies emailed, 0 sponsor money conversations</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>Active standard</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>24 Sep 2026</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>Targeting</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>Prioritise companies that already pay for film festivals, Bollywood awards or Cannes, or are entering India with money. De-prioritise AI startups and hardware giants.</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>Startup replies cite no budget (Wonder, Cascadeur, Ideogram, Hedra). Hardware majors decline via support desks.</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>New 70-company list built on this rule (WAIFF_70_Targets_Sep24.xlsx)</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>Active standard</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>24 Sep 2026</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>Organizer definition</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>Organizers = companies whose business is events or festival IP (Serendipity, Teamwork Arts, STIR, IndiaJoy, BTS, AIM). Not industrial groups.</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>MRF: 'doesn't fit into our plans'. Tyre, steel and pharma company secretaries were asked to pay EUR50k.</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>20 organizer candidates rebuilt</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>Active standard</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>24 Sep 2026</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>Message errors</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>Check merge fields. Remove false urgency, 'Apple Global', the Cannes Film Festival venue line and long AI-toned replies.</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>'Cascadeur's India edition' merge bug (13-14 Sep). Hedra CEO flagged an AI-written reply. 1,500-word Kimi rebuttal.</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>Templates rewritten (Templates sheet)</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>Active standard</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>24 Sep 2026</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>Follow-through</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>Reply to every human answer within 24h, before any new outreach.</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>NESCO (22 Sep), Cascadeur (14 Sep), Getty (11 Sep), Novotel (18 Sep), Trident (11 Sep) were left unanswered.</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>Warm-leads sheet created</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>Active standard</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>24 Sep 2026</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>Credibility</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>Ask WAiFF HQ for an @worldaifilmfestival.com mailbox and an appointment letter.</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>Personal gmail.com is rejected by many B2B forms and weakens trust with big brands.</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>Pending Aditya / Marco</t>
+        </is>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>24 Sep 2026</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>DNC compliance</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>Stop contacting existing WAiFF partners (TF1, Fnac, Station F, CapCut, MiniMax, CloudWalk/Brazil).</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>All were emailed between 13 and 19 Sep.</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>Flagged in the follow-up audit as C</t>
+        </is>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>Active standard</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>